<commit_message>
Use the Word letterhead and /notice-<id> links.
Public notices and notice emails show the rendered Being Vakil stationery and stamp. The demand letter and short email fill from each recipient, and the bank name comes from that record.

Co-authored-by: B V Solutions <akshayrsat@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/notice-recipients.xlsx
+++ b/samples/notice-recipients.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
   <si>
     <t>Customer name</t>
   </si>
@@ -40,6 +40,21 @@
     <t>Outstanding amount</t>
   </si>
   <si>
+    <t>Loan type</t>
+  </si>
+  <si>
+    <t>Reference number</t>
+  </si>
+  <si>
+    <t>Collection manager</t>
+  </si>
+  <si>
+    <t>Collection manager mobile</t>
+  </si>
+  <si>
+    <t>Bank website</t>
+  </si>
+  <si>
     <t>Co-borrower name</t>
   </si>
   <si>
@@ -70,12 +85,18 @@
     <t>akshayrsathe@gmail.com</t>
   </si>
   <si>
+    <t>14, Shivaji Nagar, Pune 411005</t>
+  </si>
+  <si>
     <t>LN10021</t>
   </si>
   <si>
     <t>CUST501</t>
   </si>
   <si>
+    <t>Home Loan</t>
+  </si>
+  <si>
     <t>Akshay R Sathe</t>
   </si>
   <si>
@@ -85,12 +106,18 @@
     <t>akshayrsat@gmail.com</t>
   </si>
   <si>
+    <t>22, Law College Road, Pune 411004</t>
+  </si>
+  <si>
     <t>LN10022</t>
   </si>
   <si>
     <t>CUST502</t>
   </si>
   <si>
+    <t>Personal Loan</t>
+  </si>
+  <si>
     <t>Shweta Sudhir</t>
   </si>
   <si>
@@ -100,10 +127,16 @@
     <t>advshwetasudhir@gmail.com</t>
   </si>
   <si>
+    <t>8, FC Road, Pune 411004</t>
+  </si>
+  <si>
     <t>LN10023</t>
   </si>
   <si>
     <t>CUST503</t>
+  </si>
+  <si>
+    <t>Housing Loan</t>
   </si>
 </sst>
 </file>
@@ -484,13 +517,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="15" width="24" customWidth="1"/>
+    <col min="1" max="20" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -536,28 +569,43 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -566,45 +614,60 @@
         <v>125000</v>
       </c>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="K2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="O2" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="P2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R2" t="s">
+        <v>22</v>
+      </c>
+      <c r="S2" t="s">
+        <v>22</v>
+      </c>
+      <c r="T2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="H3">
         <v>250000</v>
@@ -613,45 +676,60 @@
         <v>80000</v>
       </c>
       <c r="J3" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="O3" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="P3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H4">
         <v>750000</v>
@@ -660,22 +738,37 @@
         <v>210000</v>
       </c>
       <c r="J4" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="K4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="O4" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="P4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>22</v>
+      </c>
+      <c r="R4" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add personalized A4 public notices with firm letterhead
Public notice pages use Word letterhead, advocate stamp, and A4 print size. SMS/email links use notice.beingvakil.in/notice-<id>. MSG91_LIVE_SEND stays off.
</commit_message>
<xml_diff>
--- a/samples/notice-recipients.xlsx
+++ b/samples/notice-recipients.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
   <si>
     <t>Customer name</t>
   </si>
@@ -40,6 +40,21 @@
     <t>Outstanding amount</t>
   </si>
   <si>
+    <t>Loan type</t>
+  </si>
+  <si>
+    <t>Reference number</t>
+  </si>
+  <si>
+    <t>Collection manager</t>
+  </si>
+  <si>
+    <t>Collection manager mobile</t>
+  </si>
+  <si>
+    <t>Bank website</t>
+  </si>
+  <si>
     <t>Co-borrower name</t>
   </si>
   <si>
@@ -70,12 +85,18 @@
     <t>akshayrsathe@gmail.com</t>
   </si>
   <si>
+    <t>14, Shivaji Nagar, Pune 411005</t>
+  </si>
+  <si>
     <t>LN10021</t>
   </si>
   <si>
     <t>CUST501</t>
   </si>
   <si>
+    <t>Home Loan</t>
+  </si>
+  <si>
     <t>Akshay R Sathe</t>
   </si>
   <si>
@@ -85,12 +106,18 @@
     <t>akshayrsat@gmail.com</t>
   </si>
   <si>
+    <t>22, Law College Road, Pune 411004</t>
+  </si>
+  <si>
     <t>LN10022</t>
   </si>
   <si>
     <t>CUST502</t>
   </si>
   <si>
+    <t>Personal Loan</t>
+  </si>
+  <si>
     <t>Shweta Sudhir</t>
   </si>
   <si>
@@ -100,10 +127,16 @@
     <t>advshwetasudhir@gmail.com</t>
   </si>
   <si>
+    <t>8, FC Road, Pune 411004</t>
+  </si>
+  <si>
     <t>LN10023</t>
   </si>
   <si>
     <t>CUST503</t>
+  </si>
+  <si>
+    <t>Housing Loan</t>
   </si>
 </sst>
 </file>
@@ -484,13 +517,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="15" width="24" customWidth="1"/>
+    <col min="1" max="20" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -536,28 +569,43 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -566,45 +614,60 @@
         <v>125000</v>
       </c>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="K2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="O2" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="P2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R2" t="s">
+        <v>22</v>
+      </c>
+      <c r="S2" t="s">
+        <v>22</v>
+      </c>
+      <c r="T2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="H3">
         <v>250000</v>
@@ -613,45 +676,60 @@
         <v>80000</v>
       </c>
       <c r="J3" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="O3" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="P3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H4">
         <v>750000</v>
@@ -660,22 +738,37 @@
         <v>210000</v>
       </c>
       <c r="J4" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="K4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="O4" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="P4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>22</v>
+      </c>
+      <c r="R4" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>